<commit_message>
added auto-scrolls ,updtae docs
</commit_message>
<xml_diff>
--- a/reports/test-results.xlsx
+++ b/reports/test-results.xlsx
@@ -32,7 +32,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -42,11 +42,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E6F4EA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE8E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,11 +57,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -469,10 +463,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C2" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -488,13 +482,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -511,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,73 +527,73 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RBAC</t>
+          <t>Threaded chat</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tool execution</t>
+          <t>Core challenge</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Threaded chat</t>
+          <t>Persistence</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Core challenge</t>
+          <t>RBAC</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Persistence</t>
+          <t>Tool execution</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Multi-step reasoning</t>
+          <t>Execution trace</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Execution trace</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -609,31 +603,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Admin workflow</t>
+          <t>Multi-step reasoning</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Text tool</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Error handling</t>
+          <t>Admin workflow</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
@@ -643,23 +637,23 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Retry logic</t>
+          <t>Frontend workspace</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>Error handling</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -669,7 +663,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Text tool</t>
+          <t>Retry logic</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -679,7 +673,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Tool routing</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -689,7 +683,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Frontend workspace</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -699,27 +693,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Calculator tool</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Weather tool</t>
+          <t>Frontend routing</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Currency tool</t>
+          <t>Calculator tool</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -729,7 +723,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Transaction categorizer</t>
+          <t>Weather tool</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -739,7 +733,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Frontend streaming</t>
+          <t>Currency tool</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -749,7 +743,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Composer validation</t>
+          <t>Transaction categorizer</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -759,7 +753,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Frontend routing</t>
+          <t>Frontend streaming</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -769,7 +763,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Frontend admin</t>
+          <t>Composer validation</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -779,17 +773,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Core API</t>
+          <t>Frontend admin</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Health endpoint</t>
+          <t>Core API</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -799,7 +793,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Health endpoint</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -809,7 +803,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>User management</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -819,7 +813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>History search</t>
+          <t>User management</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -829,7 +823,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Deletion</t>
+          <t>History search</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -839,7 +833,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Tool routing</t>
+          <t>Deletion</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -903,6 +897,16 @@
         </is>
       </c>
       <c r="B39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Interaction polish</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
         <v>1</v>
       </c>
     </row>
@@ -917,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -995,7 +999,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.779</t>
+          <t>0.279</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -1033,7 +1037,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.758</t>
+          <t>0.516</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -1071,7 +1075,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1.360</t>
+          <t>0.873</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -1109,7 +1113,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1.416</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1117,7 +1121,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tests.integration.test_api::test_thread_can_be_deleted</t>
+          <t>tests.integration.test_api::test_api_rejects_sixth_thread</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1127,17 +1131,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>test_thread_can_be_deleted</t>
+          <t>test_api_rejects_sixth_thread</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Deleting a thread removes its stored turns and hides it from history.</t>
+          <t>Creating a sixth thread is rejected before persistence with the configured per-user chat limit.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Threaded chat, Persistence, Deletion</t>
+          <t>Threaded chat, Validation, Persistence</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1147,7 +1151,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1.338</t>
+          <t>0.553</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1155,7 +1159,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tests.integration.test_api::test_api_supports_two_subtasks_in_one_request</t>
+          <t>tests.integration.test_api::test_api_rejects_fourth_thread_flow_before_execution</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1165,17 +1169,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>test_api_supports_two_subtasks_in_one_request</t>
+          <t>test_api_rejects_fourth_thread_flow_before_execution</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>The task API supports up to two subtasks in one request and returns combined multi-tool output.</t>
+          <t>Submitting a fourth saved task flow in one chat is rejected before task execution begins.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Multi-step reasoning, Tool execution, Core challenge</t>
+          <t>Threaded chat, Validation, Execution trace</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1185,7 +1189,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.827</t>
+          <t>0.541</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1193,7 +1197,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tests.integration.test_api::test_api_rejects_more_than_two_subtasks</t>
+          <t>tests.integration.test_api::test_api_rejects_fourth_thread_flow_on_stream_route</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1203,17 +1207,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>test_api_rejects_more_than_two_subtasks</t>
+          <t>test_api_rejects_fourth_thread_flow_on_stream_route</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Requests containing more than two subtasks are rejected with a validation error.</t>
+          <t>The streaming task endpoint rejects a fourth task flow before opening an SSE execution stream.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Validation, Core challenge</t>
+          <t>Streaming, Validation, Threaded chat</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1223,7 +1227,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1.011</t>
+          <t>0.524</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1231,7 +1235,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tests.integration.test_api::test_api_returns_handled_response_for_unsupported_tasks</t>
+          <t>tests.integration.test_api::test_thread_can_be_deleted</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1241,17 +1245,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>test_api_returns_handled_response_for_unsupported_tasks</t>
+          <t>test_thread_can_be_deleted</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Unsupported requests are returned as handled task results instead of crashing the API.</t>
+          <t>Deleting a thread removes its stored turns and hides it from history.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Error handling, Unsupported task UX</t>
+          <t>Threaded chat, Persistence, Deletion</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1261,7 +1265,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.900</t>
+          <t>0.644</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -1269,7 +1273,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>tests.integration.test_api::test_api_streams_trace_steps_and_returns_completed_thread</t>
+          <t>tests.integration.test_api::test_api_supports_two_subtasks_in_one_request</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1279,17 +1283,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>test_api_streams_trace_steps_and_returns_completed_thread</t>
+          <t>test_api_supports_two_subtasks_in_one_request</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Streaming execution emits ordered trace events and finishes with the persisted thread payload.</t>
+          <t>The task API supports up to two subtasks in one request and returns combined multi-tool output.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Streaming, Execution trace, Persistence</t>
+          <t>Multi-step reasoning, Tool execution, Core challenge</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1299,7 +1303,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.696</t>
+          <t>0.588</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1307,7 +1311,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tests.integration.test_api::test_api_streams_handled_unsupported_task_turn</t>
+          <t>tests.integration.test_api::test_api_rejects_more_than_two_subtasks</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1317,17 +1321,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>test_api_streams_handled_unsupported_task_turn</t>
+          <t>test_api_rejects_more_than_two_subtasks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Streaming execution returns a completed unsupported-task turn rather than failing the stream.</t>
+          <t>Requests containing more than two subtasks are rejected with a validation error.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Streaming, Unsupported task UX</t>
+          <t>Validation, Core challenge</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1337,7 +1341,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.611</t>
+          <t>0.503</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1345,7 +1349,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>tests.integration.test_api::test_api_streams_visible_retry_before_success</t>
+          <t>tests.integration.test_api::test_api_returns_handled_response_for_unsupported_tasks</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1355,17 +1359,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>test_api_streams_visible_retry_before_success</t>
+          <t>test_api_returns_handled_response_for_unsupported_tasks</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Streaming execution surfaces retry scheduling before completing successfully after a transient tool failure.</t>
+          <t>Unsupported requests are returned as handled task results instead of crashing the API.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Streaming, Retry logic, Execution trace</t>
+          <t>Error handling, Unsupported task UX</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1375,7 +1379,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0.993</t>
+          <t>0.366</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1383,27 +1387,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_interpreter_routes_all_primary_tools</t>
+          <t>tests.integration.test_api::test_api_streams_trace_steps_and_returns_completed_thread</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent</t>
+          <t>tests.integration.test_api</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>test_interpreter_routes_all_primary_tools</t>
+          <t>test_api_streams_trace_steps_and_returns_completed_thread</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Interpreter routing selects the correct primary tool for each supported request family.</t>
+          <t>Streaming execution emits ordered trace events and finishes with the persisted thread payload.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Tool routing, Core challenge</t>
+          <t>Streaming, Execution trace, Persistence</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1413,7 +1417,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.352</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
@@ -1421,27 +1425,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_interpreter_builds_two_step_transaction_and_currency_plan</t>
+          <t>tests.integration.test_api::test_api_streams_handled_unsupported_task_turn</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent</t>
+          <t>tests.integration.test_api</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>test_interpreter_builds_two_step_transaction_and_currency_plan</t>
+          <t>test_api_streams_handled_unsupported_task_turn</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Interpreter builds the chained categorization-to-currency plan for supported finance prompts.</t>
+          <t>Streaming execution returns a completed unsupported-task turn rather than failing the stream.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Multi-step reasoning, Planning</t>
+          <t>Streaming, Unsupported task UX</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1451,7 +1455,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.331</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1459,27 +1463,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_interpreter_builds_two_independent_subtasks_from_natural_language</t>
+          <t>tests.integration.test_api::test_api_streams_visible_retry_before_success</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent</t>
+          <t>tests.integration.test_api</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>test_interpreter_builds_two_independent_subtasks_from_natural_language</t>
+          <t>test_api_streams_visible_retry_before_success</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Interpreter splits supported natural-language requests into two independent tool steps.</t>
+          <t>Streaming execution surfaces retry scheduling before completing successfully after a transient tool failure.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Multi-step reasoning, Planning</t>
+          <t>Streaming, Retry logic, Execution trace</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1489,7 +1493,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.318</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
@@ -1497,7 +1501,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_interpreter_supports_unquoted_text_task_in_multi_subtask_mode</t>
+          <t>tests.unit.test_agent::test_interpreter_routes_all_primary_tools</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1507,17 +1511,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>test_interpreter_supports_unquoted_text_task_in_multi_subtask_mode</t>
+          <t>test_interpreter_routes_all_primary_tools</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Interpreter accepts unquoted text transforms inside a two-subtask request.</t>
+          <t>Interpreter routing selects the correct primary tool for each supported request family.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Multi-step reasoning, Text tool</t>
+          <t>Tool routing, Core challenge</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1535,7 +1539,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_interpreter_rejects_more_than_two_subtasks</t>
+          <t>tests.unit.test_agent::test_interpreter_routes_supported_synonym_prompts</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1545,17 +1549,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>test_interpreter_rejects_more_than_two_subtasks</t>
+          <t>test_interpreter_routes_supported_synonym_prompts</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Interpreter enforces the maximum of two subtasks per request.</t>
+          <t>Interpreter recognizes the documented natural-language synonym prompts for text, calculator, weather, currency, and transaction tools.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Validation, Planning</t>
+          <t>Tool routing, Core challenge, Validation</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1573,7 +1577,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_controller_combines_multi_subtask_results</t>
+          <t>tests.unit.test_agent::test_interpreter_builds_two_step_transaction_and_currency_plan</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1583,17 +1587,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>test_controller_combines_multi_subtask_results</t>
+          <t>test_interpreter_builds_two_step_transaction_and_currency_plan</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Controller combines multiple tool outputs into one ordered final response payload.</t>
+          <t>Interpreter builds the chained categorization-to-currency plan for supported finance prompts.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Execution trace, Multi-step reasoning, Core challenge</t>
+          <t>Multi-step reasoning, Planning</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1611,7 +1615,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_controller_returns_handled_unsupported_turn</t>
+          <t>tests.unit.test_agent::test_interpreter_builds_two_independent_subtasks_from_natural_language</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1621,17 +1625,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>test_controller_returns_handled_unsupported_turn</t>
+          <t>test_interpreter_builds_two_independent_subtasks_from_natural_language</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Controller converts unsupported requests into handled thread turns with response assembly steps.</t>
+          <t>Interpreter splits supported natural-language requests into two independent tool steps.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Error handling, Unsupported task UX</t>
+          <t>Multi-step reasoning, Planning</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1649,7 +1653,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_controller_retries_retryable_tool_failures_once</t>
+          <t>tests.unit.test_agent::test_interpreter_supports_unquoted_text_task_in_multi_subtask_mode</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1659,17 +1663,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>test_controller_retries_retryable_tool_failures_once</t>
+          <t>test_interpreter_supports_unquoted_text_task_in_multi_subtask_mode</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Controller retries a retryable tool failure once and records the retry step in the trace.</t>
+          <t>Interpreter accepts unquoted text transforms inside a two-subtask request.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Retry logic, Execution trace</t>
+          <t>Multi-step reasoning, Text tool</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1687,7 +1691,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_controller_returns_failed_turn_when_retryable_error_keeps_failing</t>
+          <t>tests.unit.test_agent::test_interpreter_rejects_more_than_two_subtasks</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1697,17 +1701,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>test_controller_returns_failed_turn_when_retryable_error_keeps_failing</t>
+          <t>test_interpreter_rejects_more_than_two_subtasks</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Controller returns a handled failed turn when a retryable tool error still fails after the retry limit.</t>
+          <t>Interpreter enforces the maximum of two subtasks per request.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Retry logic, Error handling</t>
+          <t>Validation, Planning</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1717,7 +1721,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1725,7 +1729,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_repository_seeds_default_users</t>
+          <t>tests.unit.test_agent::test_controller_combines_multi_subtask_results</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1735,17 +1739,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>test_repository_seeds_default_users</t>
+          <t>test_controller_combines_multi_subtask_results</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Repository initialization seeds only the documented bootstrap admin account.</t>
+          <t>Controller combines multiple tool outputs into one ordered final response payload.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>RBAC, Persistence, Setup</t>
+          <t>Execution trace, Multi-step reasoning, Core challenge</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1755,7 +1759,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0.654</t>
+          <t>0.013</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1763,7 +1767,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_thread_persists_masked_turns_and_auto_titles</t>
+          <t>tests.unit.test_agent::test_controller_counts_words_for_count_the_word_prompt</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1773,17 +1777,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>test_thread_persists_masked_turns_and_auto_titles</t>
+          <t>test_controller_counts_words_for_count_the_word_prompt</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Repository persists masked turn content and auto-generates thread titles from the first task.</t>
+          <t>Controller treats count-the-word prompts as supported text word-count requests and returns the expected completed output.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Persistence, Safety, Threaded chat</t>
+          <t>Text tool, Core challenge, Tool routing</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1793,7 +1797,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.553</t>
+          <t>0.012</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -1801,7 +1805,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_repository_enforces_password_policy_for_created_users</t>
+          <t>tests.unit.test_agent::test_controller_returns_handled_unsupported_turn</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1811,17 +1815,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>test_repository_enforces_password_policy_for_created_users</t>
+          <t>test_controller_returns_handled_unsupported_turn</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Repository rejects new users whose passwords do not meet the documented policy.</t>
+          <t>Controller converts unsupported requests into handled thread turns with response assembly steps.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Admin workflow, Validation, RBAC</t>
+          <t>Error handling, Unsupported task UX</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1831,7 +1835,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0.623</t>
+          <t>0.013</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1839,7 +1843,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>tests.unit.test_agent::test_repository_enforces_role_limits_for_created_users</t>
+          <t>tests.unit.test_agent::test_controller_returns_handled_unsupported_turn_for_occurrence_count_prompt</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1849,17 +1853,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>test_repository_enforces_role_limits_for_created_users</t>
+          <t>test_controller_returns_handled_unsupported_turn_for_occurrence_count_prompt</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Repository enforces the configured maximum number of admin and standard user accounts.</t>
+          <t>Controller keeps substring or occurrence-count wording unsupported and returns a handled unsupported-task turn.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Admin workflow, RBAC, Validation</t>
+          <t>Text tool, Unsupported task UX, Validation</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1869,7 +1873,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>0.720</t>
+          <t>0.012</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -1877,27 +1881,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>tests.unit.test_safety::test_safety_guard_rejects_more_than_two_hundred_fifty_characters</t>
+          <t>tests.unit.test_agent::test_controller_retries_retryable_tool_failures_once</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>tests.unit.test_safety</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>test_safety_guard_rejects_more_than_two_hundred_fifty_characters</t>
+          <t>test_controller_retries_retryable_tool_failures_once</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Safety guard rejects input longer than the documented 250 character limit.</t>
+          <t>Controller retries a retryable tool failure once and records the retry step in the trace.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Safety, Validation</t>
+          <t>Retry logic, Execution trace</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1907,7 +1911,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.013</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -1915,27 +1919,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>tests.unit.test_safety::test_safety_guard_accepts_exactly_two_hundred_fifty_characters</t>
+          <t>tests.unit.test_agent::test_controller_returns_failed_turn_when_retryable_error_keeps_failing</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>tests.unit.test_safety</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>test_safety_guard_accepts_exactly_two_hundred_fifty_characters</t>
+          <t>test_controller_returns_failed_turn_when_retryable_error_keeps_failing</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Safety guard accepts input that is exactly at the documented character limit.</t>
+          <t>Controller returns a handled failed turn when a retryable tool error still fails after the retry limit.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Safety, Validation</t>
+          <t>Retry logic, Error handling</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1945,7 +1949,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.013</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1953,27 +1957,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_text_processor_uppercase</t>
+          <t>tests.unit.test_agent::test_repository_seeds_default_users</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>test_text_processor_uppercase</t>
+          <t>test_repository_seeds_default_users</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Text processor returns uppercase output for supported requests.</t>
+          <t>Repository initialization seeds only the documented bootstrap admin account.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Text tool, Tool execution</t>
+          <t>RBAC, Persistence, Setup</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1983,7 +1987,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.252</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -1991,27 +1995,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_text_processor_missing_text</t>
+          <t>tests.unit.test_agent::test_thread_persists_masked_turns_and_auto_titles</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>test_text_processor_missing_text</t>
+          <t>test_thread_persists_masked_turns_and_auto_titles</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Text processor rejects requests that omit the required text target.</t>
+          <t>Repository persists masked turn content and auto-generates thread titles from the first task.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Text tool, Validation</t>
+          <t>Persistence, Safety, Threaded chat</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2021,7 +2025,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.174</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -2029,27 +2033,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_calculator_precedence</t>
+          <t>tests.unit.test_agent::test_repository_enforces_password_policy_for_created_users</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>test_calculator_precedence</t>
+          <t>test_repository_enforces_password_policy_for_created_users</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Calculator preserves arithmetic precedence and parentheses order.</t>
+          <t>Repository rejects new users whose passwords do not meet the documented policy.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Calculator tool, Tool execution</t>
+          <t>Admin workflow, Validation, RBAC</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2059,7 +2063,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.143</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -2067,27 +2071,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_calculator_divide_by_zero</t>
+          <t>tests.unit.test_agent::test_repository_enforces_role_limits_for_created_users</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>test_calculator_divide_by_zero</t>
+          <t>test_repository_enforces_role_limits_for_created_users</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Calculator rejects divide-by-zero expressions safely.</t>
+          <t>Repository enforces the configured maximum number of admin and standard user accounts.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Calculator tool, Validation</t>
+          <t>Admin workflow, RBAC, Validation</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2097,7 +2101,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.480</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -2105,27 +2109,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_weather_city_is_case_insensitive</t>
+          <t>tests.unit.test_agent::test_repository_enforces_thread_limit</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>test_weather_city_is_case_insensitive</t>
+          <t>test_repository_enforces_thread_limit</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Weather tool matches supported cities without case sensitivity.</t>
+          <t>Repository rejects a sixth chat thread for the same user.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Weather tool, Tool execution</t>
+          <t>Threaded chat, Validation, Persistence</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2135,7 +2139,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.178</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -2143,27 +2147,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_weather_rejects_unsupported_city</t>
+          <t>tests.unit.test_agent::test_repository_enforces_thread_flow_limit</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_agent</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>test_weather_rejects_unsupported_city</t>
+          <t>test_repository_enforces_thread_flow_limit</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Weather tool returns a validation error when the city is outside the supported mock list.</t>
+          <t>Repository rejects a fourth saved task flow inside the same chat thread.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Weather tool, Validation</t>
+          <t>Threaded chat, Validation, Persistence</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2173,7 +2177,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.210</t>
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
@@ -2181,29 +2185,25 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_currency_converter_converts_between_supported_codes</t>
+          <t>tests.unit.test_reports::test_normalize_coverage_label_strips_bonus_prefix</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_reports</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>test_currency_converter_converts_between_supported_codes</t>
+          <t>test_normalize_coverage_label_strips_bonus_prefix</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Currency converter returns the expected converted amount for supported codes.</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Currency tool, Tool execution</t>
-        </is>
-      </c>
+          <t>test normalize coverage label strips bonus prefix</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>passed</t>
@@ -2219,29 +2219,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_currency_converter_rejects_negative_amount</t>
+          <t>tests.unit.test_reports::test_parse_junit_normalizes_coverage_labels</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_reports</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>test_currency_converter_rejects_negative_amount</t>
+          <t>test_parse_junit_normalizes_coverage_labels</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Currency converter rejects negative amounts.</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Currency tool, Validation</t>
-        </is>
-      </c>
+          <t>test parse junit normalizes coverage labels</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
           <t>passed</t>
@@ -2249,7 +2245,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.005</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
@@ -2257,29 +2253,25 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools::test_transaction_categorizer_matches_keywords</t>
+          <t>tests.unit.test_reports::test_build_dashboard_omits_bonus_prefix_from_rendered_html</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>tests.unit.test_tools</t>
+          <t>tests.unit.test_reports</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>test_transaction_categorizer_matches_keywords</t>
+          <t>test_build_dashboard_omits_bonus_prefix_from_rendered_html</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Transaction categorizer matches merchant keywords to the expected spending category.</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Transaction categorizer, Tool execution</t>
-        </is>
-      </c>
+          <t>test build dashboard omits bonus prefix from rendered html</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr">
         <is>
           <t>passed</t>
@@ -2295,40 +2287,458 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>tests.unit.test_safety::test_safety_guard_rejects_more_than_two_hundred_fifty_characters</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>tests.unit.test_safety</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>test_safety_guard_rejects_more_than_two_hundred_fifty_characters</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Safety guard rejects input longer than the documented 250 character limit.</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Safety, Validation</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>tests.unit.test_safety::test_safety_guard_accepts_exactly_two_hundred_fifty_characters</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>tests.unit.test_safety</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>test_safety_guard_accepts_exactly_two_hundred_fifty_characters</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Safety guard accepts input that is exactly at the documented character limit.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Safety, Validation</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_text_processor_uppercase</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>test_text_processor_uppercase</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Text processor returns uppercase output for supported requests.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Text tool, Tool execution</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_text_processor_missing_text</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>test_text_processor_missing_text</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Text processor rejects requests that omit the required text target.</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Text tool, Validation</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_calculator_precedence</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>test_calculator_precedence</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Calculator preserves arithmetic precedence and parentheses order.</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Calculator tool, Tool execution</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_calculator_divide_by_zero</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>test_calculator_divide_by_zero</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Calculator rejects divide-by-zero expressions safely.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Calculator tool, Validation</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_weather_city_is_case_insensitive</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>test_weather_city_is_case_insensitive</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Weather tool matches supported cities without case sensitivity.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Weather tool, Tool execution</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_weather_rejects_unsupported_city</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>test_weather_rejects_unsupported_city</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Weather tool returns a validation error when the city is outside the supported mock list.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Weather tool, Validation</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_currency_converter_converts_between_supported_codes</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>test_currency_converter_converts_between_supported_codes</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Currency converter returns the expected converted amount for supported codes.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Currency tool, Tool execution</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_currency_converter_rejects_negative_amount</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>test_currency_converter_rejects_negative_amount</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Currency converter rejects negative amounts.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Currency tool, Validation</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools::test_transaction_categorizer_matches_keywords</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>tests.unit.test_tools</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>test_transaction_categorizer_matches_keywords</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Transaction categorizer matches merchant keywords to the expected spending category.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Transaction categorizer, Tool execution</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>tests.unit.test_tools::test_transaction_categorizer_falls_back_to_other</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>tests.unit.test_tools</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>test_transaction_categorizer_falls_back_to_other</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Transaction categorizer falls back to the generic other category when no keyword matches.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Transaction categorizer, Tool execution</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
         <is>
           <t>0.002</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2341,7 +2751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2419,7 +2829,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.3286077</t>
+          <t>0.3832605</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -2450,29 +2860,22 @@
           <t>Frontend workspace, Core challenge, Response hierarchy</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>failed</t>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.2722468</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>expected '/' to be '/threads/thread-2' // Object.is equality AssertionError: expected '/' to be '/threads/thread-2' // Object.is equality
-Expected: "/threads/thread-2"
-Received: "/"
- ❯ src/App.test.tsx:332:38</t>
-        </is>
-      </c>
+          <t>0.3510417</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; renders streamed execution trace steps before completion</t>
+          <t>src/App.test.tsx::App &gt; creates a chat from the home workspace on first submission and activates the thread route</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2482,17 +2885,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>App &gt; renders streamed execution trace steps before completion</t>
+          <t>App &gt; creates a chat from the home workspace on first submission and activates the thread route</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The workspace shows streamed trace steps live before the final persisted turn replaces the pending card.</t>
+          <t>Submitting the first task from workspace home creates a new chat and activates the thread route using the created thread payload.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Frontend streaming, Execution trace, Streaming</t>
+          <t>Frontend routing, Threaded chat, Core challenge</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -2502,7 +2905,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.3667808</t>
+          <t>0.2013687</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -2510,7 +2913,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; falls back to synchronous submission when streaming is unavailable</t>
+          <t>src/App.test.tsx::App &gt; renders streamed execution trace steps before completion</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2520,17 +2923,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>App &gt; falls back to synchronous submission when streaming is unavailable</t>
+          <t>App &gt; renders streamed execution trace steps before completion</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>The frontend falls back to the synchronous task endpoint when streaming cannot be established.</t>
+          <t>The workspace shows streamed trace steps live before the final persisted turn replaces the pending card.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Frontend streaming, Fallback behavior</t>
+          <t>Frontend streaming, Execution trace, Streaming</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2540,7 +2943,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.1741088</t>
+          <t>0.450278</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -2548,7 +2951,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; collapses and expands the history panel from the rail</t>
+          <t>src/App.test.tsx::App &gt; falls back to synchronous submission when streaming is unavailable</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2558,17 +2961,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>App &gt; collapses and expands the history panel from the rail</t>
+          <t>App &gt; falls back to synchronous submission when streaming is unavailable</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The left rail toggle collapses and re-expands the thread history panel without breaking workspace access.</t>
+          <t>The frontend falls back to the synchronous task endpoint when streaming cannot be established.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Frontend workspace, History sidebar</t>
+          <t>Frontend streaming, Fallback behavior</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2578,7 +2981,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.1000948</t>
+          <t>0.1664482</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -2586,7 +2989,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; shows inline composer validation for too many subtasks</t>
+          <t>src/App.test.tsx::App &gt; collapses and expands the history panel from the rail</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2596,17 +2999,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>App &gt; shows inline composer validation for too many subtasks</t>
+          <t>App &gt; collapses and expands the history panel from the rail</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Composer validation appears inline when a request exceeds the two-subtask limit.</t>
+          <t>The left rail toggle collapses and re-expands the thread history panel without breaking workspace access.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Composer validation, Core challenge</t>
+          <t>Frontend workspace, History sidebar</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2616,7 +3019,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0.0771534</t>
+          <t>0.1142635</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -2624,7 +3027,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; loads direct thread routes and redirects missing threads home</t>
+          <t>src/App.test.tsx::App &gt; shows inline composer validation for too many subtasks</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2634,17 +3037,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>App &gt; loads direct thread routes and redirects missing threads home</t>
+          <t>App &gt; shows inline composer validation for too many subtasks</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Direct thread URLs resolve to a saved chat or redirect back to the home workspace when the thread is missing.</t>
+          <t>Composer validation appears inline when a request exceeds the two-subtask limit.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Frontend routing, Threaded chat, Validation</t>
+          <t>Composer validation, Core challenge</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2654,7 +3057,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.0705427</t>
+          <t>0.0807562</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -2662,7 +3065,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; blocks creating a sixth thread from the sidebar</t>
+          <t>src/App.test.tsx::App &gt; loads direct thread routes and redirects missing threads home</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2672,17 +3075,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>App &gt; blocks creating a sixth thread from the sidebar</t>
+          <t>App &gt; loads direct thread routes and redirects missing threads home</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>The sidebar disables new chat creation when the user has already reached the five-thread limit.</t>
+          <t>Direct thread URLs resolve to a saved chat or redirect back to the home workspace when the thread is missing.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Frontend workspace, Validation, Threaded chat</t>
+          <t>Frontend routing, Threaded chat, Validation</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -2692,7 +3095,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.1135684</t>
+          <t>0.0572637</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -2700,7 +3103,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; blocks submissions when a chat already has three task flows</t>
+          <t>src/App.test.tsx::App &gt; blocks creating a sixth thread from the sidebar</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2710,17 +3113,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>App &gt; blocks submissions when a chat already has three task flows</t>
+          <t>App &gt; blocks creating a sixth thread from the sidebar</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>The composer is disabled when the selected chat already contains three saved task flows.</t>
+          <t>The sidebar disables new chat creation when the user has already reached the five-thread limit.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Composer validation, Threaded chat, Frontend routing</t>
+          <t>Frontend workspace, Validation, Threaded chat</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -2730,7 +3133,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.1372259</t>
+          <t>0.1084234</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -2738,7 +3141,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>src/App.test.tsx::App &gt; navigates to the admin page and reveals passwords only for session-created users</t>
+          <t>src/App.test.tsx::App &gt; blocks submissions when a chat already has three task flows</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2748,17 +3151,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>App &gt; navigates to the admin page and reveals passwords only for session-created users</t>
+          <t>App &gt; blocks submissions when a chat already has three task flows</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Admins can open the admin page, create users, reveal passwords only for users created in the current session, and delete those users.</t>
+          <t>The composer is disabled when the selected chat already contains three saved task flows.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Admin workflow, RBAC, Frontend admin</t>
+          <t>Composer validation, Threaded chat, Frontend routing</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -2768,7 +3171,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0.4371495</t>
+          <t>0.1285028</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -2776,40 +3179,116 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>src/App.test.tsx::App &gt; auto-scrolls the active thread when a later response is appended</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>src/App.test.tsx</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>App &gt; auto-scrolls the active thread when a later response is appended</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>The active chat auto-scrolls to the newest pending and completed content when a later response is appended in-session.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Frontend workspace, Threaded chat, Interaction polish</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.2167385</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>src/App.test.tsx::App &gt; navigates to the admin page and reveals passwords only for session-created users</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>src/App.test.tsx</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>App &gt; navigates to the admin page and reveals passwords only for session-created users</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Admins can open the admin page, create users, reveal passwords only for users created in the current session, and delete those users.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Admin workflow, RBAC, Frontend admin</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.6857964</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>src/App.test.tsx::App &gt; keeps admin navigation hidden for standard users</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>src/App.test.tsx</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>App &gt; keeps admin navigation hidden for standard users</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Standard users do not see admin navigation controls in the workspace.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>RBAC, Frontend admin</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>0.0387839</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.0477441</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>